<commit_message>
Practiced Advanced Functions like sumif and sumifs
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -2046,8 +2046,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="169" formatCode="[$INR]\ #,##0.00"/>
-    <numFmt numFmtId="174" formatCode="[$₹-44E]#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$INR]\ #,##0.00"/>
+    <numFmt numFmtId="166" formatCode="[$₹-44E]#,##0.00"/>
   </numFmts>
   <fonts count="22" x14ac:knownFonts="1">
     <font>
@@ -2583,7 +2583,7 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2593,7 +2593,7 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="40% - Accent4" xfId="3" builtinId="43"/>

</xml_diff>

<commit_message>
Learn't about indirect function,concat,offset function
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,22 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omsup\Documents\Advanced Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFF2CC8-D5BE-42E2-801F-C051CD4465F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE7EDBCD-2659-4504-9A3E-551BBC6AE1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="cond_formatting" sheetId="1" r:id="rId1"/>
-    <sheet name="Flashfill_custom_list" sheetId="3" r:id="rId2"/>
-    <sheet name="custom_list" sheetId="4" r:id="rId3"/>
-    <sheet name="custom_list_months" sheetId="5" r:id="rId4"/>
-    <sheet name="if_else" sheetId="7" r:id="rId5"/>
-    <sheet name="Advanced_functions" sheetId="8" r:id="rId6"/>
-    <sheet name="Sheet2" sheetId="9" r:id="rId7"/>
-    <sheet name="Lookup_func" sheetId="10" r:id="rId8"/>
+    <sheet name="Indirect" sheetId="12" r:id="rId1"/>
+    <sheet name="concat" sheetId="13" r:id="rId2"/>
+    <sheet name="cond_formatting" sheetId="1" r:id="rId3"/>
+    <sheet name="Flashfill_custom_list" sheetId="3" r:id="rId4"/>
+    <sheet name="custom_list" sheetId="4" r:id="rId5"/>
+    <sheet name="custom_list_months" sheetId="5" r:id="rId6"/>
+    <sheet name="if_else" sheetId="7" r:id="rId7"/>
+    <sheet name="Advanced_functions" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet2" sheetId="9" r:id="rId9"/>
+    <sheet name="Lookup_func" sheetId="10" r:id="rId10"/>
+    <sheet name="hlookup" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet2!$C$15:$C$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Sheet2!$C$15:$C$24</definedName>
+    <definedName name="Apples">concat!$B$2:$B$6</definedName>
+    <definedName name="Bananas">concat!$C$2:$C$6</definedName>
+    <definedName name="Lemons">concat!$D$2:$D$6</definedName>
     <definedName name="orders">Table3[Order_ID]</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -40,7 +46,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId12" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
     </ext>
   </extLst>
 </workbook>
@@ -69,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4722" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4773" uniqueCount="716">
   <si>
     <t>Region</t>
   </si>
@@ -2148,6 +2154,75 @@
   </si>
   <si>
     <t>index-match</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>using vlookup</t>
+  </si>
+  <si>
+    <t>using index-match</t>
+  </si>
+  <si>
+    <t>E4</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>R2C1</t>
+  </si>
+  <si>
+    <t>R1C1 Style</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Amit</t>
+  </si>
+  <si>
+    <t>Sunil</t>
+  </si>
+  <si>
+    <t>Bananas</t>
+  </si>
+  <si>
+    <t>Lemons</t>
+  </si>
+  <si>
+    <t>Fruit:</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>using xlookup</t>
   </si>
 </sst>
 </file>
@@ -2159,11 +2234,18 @@
     <numFmt numFmtId="165" formatCode="[$INR]\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$₹-439]#,##0.00"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2314,7 +2396,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2378,6 +2460,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2585,105 +2673,106 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="10" fontId="9" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="10" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="7" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="15" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="15" fillId="7" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="15" fillId="7" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="15" fillId="7" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="16" fillId="8" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="16" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="16" fillId="7" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="16" fillId="7" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="16" fillId="7" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="17" fillId="8" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="9" fontId="17" fillId="7" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="18" fillId="7" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="9" fontId="17" fillId="7" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="18" fillId="7" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="9" fontId="18" fillId="8" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="19" fillId="8" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="18" fillId="8" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="19" fillId="8" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2692,71 +2781,68 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="16" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2765,17 +2851,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="40% - Accent4" xfId="3" builtinId="43"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="4" xr:uid="{88D63144-27FB-4D9D-A79B-725FA5FE3C0E}"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="45">
@@ -4097,6 +4190,679 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D81F403-80D2-451A-BE2B-A0BA740AF252}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="5" width="8.88671875" style="91"/>
+    <col min="6" max="6" width="11.5546875" style="91" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="91"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="91">
+        <v>111</v>
+      </c>
+      <c r="C1" s="91" t="s">
+        <v>703</v>
+      </c>
+      <c r="D1" s="91" cm="1">
+        <f t="array" aca="1" ref="D1" ca="1">INDIRECT(C1)</f>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="91">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="91">
+        <v>333</v>
+      </c>
+      <c r="C3" s="91" t="s">
+        <v>704</v>
+      </c>
+      <c r="D3" s="91" cm="1">
+        <f t="array" aca="1" ref="D3" ca="1">INDIRECT(C3,FALSE)</f>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E4" s="91">
+        <v>4</v>
+      </c>
+      <c r="F4" s="91" t="s">
+        <v>702</v>
+      </c>
+      <c r="H4" s="91" cm="1">
+        <f t="array" aca="1" ref="H4" ca="1">INDIRECT(F4)+100</f>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="92" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="92" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" s="91" t="s">
+        <v>583</v>
+      </c>
+      <c r="E12" s="91" t="s">
+        <v>549</v>
+      </c>
+      <c r="F12" s="91" t="str">
+        <f>D12&amp;"   "&amp;E12</f>
+        <v>Ankit   Sharma</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4FCD3B0-4BC8-4681-8037-4E058512B5F9}">
+  <dimension ref="B1:J19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="J1" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="85" t="s">
+        <v>686</v>
+      </c>
+      <c r="C2" s="85" t="s">
+        <v>600</v>
+      </c>
+      <c r="D2" s="85" t="s">
+        <v>577</v>
+      </c>
+      <c r="E2" s="85" t="s">
+        <v>624</v>
+      </c>
+      <c r="F2" s="85" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B3" s="25">
+        <v>1001</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>604</v>
+      </c>
+      <c r="D3" s="25">
+        <v>70000</v>
+      </c>
+      <c r="E3" s="84">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="25">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B4" s="25">
+        <v>1002</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>605</v>
+      </c>
+      <c r="D4" s="25">
+        <v>50000</v>
+      </c>
+      <c r="E4" s="84">
+        <v>0.05</v>
+      </c>
+      <c r="F4" s="25">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B5" s="25">
+        <v>1003</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>606</v>
+      </c>
+      <c r="D5" s="25">
+        <v>45000</v>
+      </c>
+      <c r="E5" s="84">
+        <v>0</v>
+      </c>
+      <c r="F5" s="25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B6" s="25">
+        <v>1004</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>607</v>
+      </c>
+      <c r="D6" s="25">
+        <v>75000</v>
+      </c>
+      <c r="E6" s="84">
+        <v>0.15</v>
+      </c>
+      <c r="F6" s="25">
+        <v>11250</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B7" s="25">
+        <v>1005</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>623</v>
+      </c>
+      <c r="D7" s="25">
+        <v>55000</v>
+      </c>
+      <c r="E7" s="84">
+        <v>0.05</v>
+      </c>
+      <c r="F7" s="25">
+        <v>2750</v>
+      </c>
+      <c r="G7" t="s">
+        <v>688</v>
+      </c>
+      <c r="H7">
+        <f>MATCH(B4,B2:B7,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="88" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="86" t="s">
+        <v>687</v>
+      </c>
+      <c r="D9" s="86" t="s">
+        <v>577</v>
+      </c>
+      <c r="E9" s="86" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="25">
+        <v>1002</v>
+      </c>
+      <c r="D10" s="25">
+        <f>VLOOKUP(C10,B2:F7,MATCH("Sales",B2:F2,0),FALSE)</f>
+        <v>50000</v>
+      </c>
+      <c r="E10" s="87">
+        <f>VLOOKUP(C10,B2:F7,MATCH("Bonus Amount",B2:F2,0),FALSE)</f>
+        <v>2500</v>
+      </c>
+      <c r="G10" t="s">
+        <v>689</v>
+      </c>
+      <c r="H10">
+        <f>MATCH("Sales",B2:F2,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="52" t="s">
+        <v>691</v>
+      </c>
+      <c r="G12" t="s">
+        <v>688</v>
+      </c>
+      <c r="I12">
+        <f>MATCH(C15,B2:B7,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>689</v>
+      </c>
+      <c r="I13">
+        <f>MATCH("Sales",B2:F2,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="89" t="s">
+        <v>687</v>
+      </c>
+      <c r="D14" s="89" t="s">
+        <v>577</v>
+      </c>
+      <c r="E14" s="89" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="25">
+        <v>1004</v>
+      </c>
+      <c r="D15" s="25">
+        <f>INDEX(B2:F7,MATCH(C15,B2:B7,0),MATCH("Sales",B2:F2,0))</f>
+        <v>75000</v>
+      </c>
+      <c r="E15" s="25">
+        <f>INDEX(B2:F7,MATCH(C15,B2:B7,0),MATCH("Bonus Amount",B2:F2,0))</f>
+        <v>11250</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C18" s="89" t="s">
+        <v>687</v>
+      </c>
+      <c r="D18" s="89" t="s">
+        <v>577</v>
+      </c>
+      <c r="E18" s="89" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C19" s="25">
+        <v>1004</v>
+      </c>
+      <c r="D19" s="25">
+        <f>_xlfn.XLOOKUP(C19,$B$3:$B$7,$D$3:$D$7)</f>
+        <v>75000</v>
+      </c>
+      <c r="E19" s="25">
+        <f>_xlfn.XLOOKUP(C19,$B$3:$B$7,$F$3:$F$7)</f>
+        <v>11250</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10" xr:uid="{A047E17B-A2CA-4FD8-92FF-2040F978D0C4}">
+      <formula1>$B$3:$B$7</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15 C19" xr:uid="{D0E06332-745C-4019-A65E-6A1EF7168DF7}">
+      <formula1>$B$2:$B$7</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBEC3E4-77E5-4A66-A09B-D9FF6175E7CC}">
+  <dimension ref="A3:H20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="25"/>
+      <c r="B3" s="26" t="s">
+        <v>693</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>694</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>695</v>
+      </c>
+      <c r="E3" s="26" t="s">
+        <v>696</v>
+      </c>
+      <c r="F3" s="26" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="26" t="s">
+        <v>697</v>
+      </c>
+      <c r="B4" s="25">
+        <v>100</v>
+      </c>
+      <c r="C4" s="25">
+        <v>585</v>
+      </c>
+      <c r="D4" s="25">
+        <v>333</v>
+      </c>
+      <c r="E4" s="25">
+        <v>745</v>
+      </c>
+      <c r="F4" s="25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
+        <v>698</v>
+      </c>
+      <c r="B5" s="25">
+        <v>100</v>
+      </c>
+      <c r="C5" s="25">
+        <v>500</v>
+      </c>
+      <c r="D5" s="25">
+        <v>600</v>
+      </c>
+      <c r="E5" s="25">
+        <v>700</v>
+      </c>
+      <c r="F5" s="25">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
+        <v>577</v>
+      </c>
+      <c r="B6" s="25">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="25">
+        <v>7000</v>
+      </c>
+      <c r="D6" s="25">
+        <v>8000</v>
+      </c>
+      <c r="E6" s="25">
+        <v>6000</v>
+      </c>
+      <c r="F6" s="25">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>699</v>
+      </c>
+      <c r="B7" s="25">
+        <v>400</v>
+      </c>
+      <c r="C7" s="25">
+        <v>500</v>
+      </c>
+      <c r="D7" s="25">
+        <v>300</v>
+      </c>
+      <c r="E7" s="25">
+        <v>300</v>
+      </c>
+      <c r="F7" s="25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F9" s="90" t="s">
+        <v>700</v>
+      </c>
+      <c r="G9" s="90"/>
+      <c r="H9">
+        <f>MATCH(C10,A3:F3,0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B10" s="90" t="s">
+        <v>586</v>
+      </c>
+      <c r="C10" s="90" t="s">
+        <v>693</v>
+      </c>
+      <c r="F10" s="90" t="s">
+        <v>586</v>
+      </c>
+      <c r="G10" s="90" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B11" s="90" t="s">
+        <v>577</v>
+      </c>
+      <c r="C11" s="28">
+        <f>HLOOKUP($C$10,$A$3:$F$7,MATCH(B11,$A$3:$A$7,0),FALSE)</f>
+        <v>2000</v>
+      </c>
+      <c r="F11" s="90" t="s">
+        <v>577</v>
+      </c>
+      <c r="G11" s="28">
+        <f>VLOOKUP(F11,$A$3:$F$7,MATCH($G$10,$A$3:$F$3,0),FALSE)</f>
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="90" t="s">
+        <v>698</v>
+      </c>
+      <c r="C12" s="28">
+        <f>HLOOKUP($C$10,$A$3:$F$7,MATCH(B12,$A$3:$A$7,0),FALSE)</f>
+        <v>100</v>
+      </c>
+      <c r="F12" s="90" t="s">
+        <v>699</v>
+      </c>
+      <c r="G12" s="28">
+        <f>VLOOKUP(F12,$A$3:$F$7,MATCH($G$10,$A$3:$F$3,0),FALSE)</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B13" s="90" t="s">
+        <v>699</v>
+      </c>
+      <c r="C13" s="28">
+        <f>HLOOKUP($C$10,$A$3:$F$7,MATCH(B13,$A$3:$A$7,0),FALSE)</f>
+        <v>400</v>
+      </c>
+      <c r="F13" s="90" t="s">
+        <v>697</v>
+      </c>
+      <c r="G13" s="28">
+        <f>VLOOKUP(F13,$A$3:$F$7,MATCH($G$10,$A$3:$F$3,0),FALSE)</f>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F16" s="90" t="s">
+        <v>701</v>
+      </c>
+      <c r="G16" s="90"/>
+    </row>
+    <row r="17" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F17" s="90" t="s">
+        <v>586</v>
+      </c>
+      <c r="G17" s="90" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="18" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F18" s="90" t="s">
+        <v>577</v>
+      </c>
+      <c r="G18" s="28"/>
+    </row>
+    <row r="19" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F19" s="90" t="s">
+        <v>699</v>
+      </c>
+      <c r="G19" s="28"/>
+    </row>
+    <row r="20" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F20" s="90" t="s">
+        <v>697</v>
+      </c>
+      <c r="G20" s="28"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10 G10 G17" xr:uid="{65F6DE29-6950-4D2F-B0EB-D3A0B82AC2CC}">
+      <formula1>$B$3:$F$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A088EC8-1CAB-4CC3-96BB-F72ABE6822D1}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="28"/>
+      <c r="B1" s="93" t="s">
+        <v>650</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>709</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>710</v>
+      </c>
+      <c r="F1" s="95" t="s">
+        <v>711</v>
+      </c>
+      <c r="G1" s="95" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="94" t="s">
+        <v>707</v>
+      </c>
+      <c r="B2" s="28">
+        <v>55</v>
+      </c>
+      <c r="C2" s="28">
+        <v>44</v>
+      </c>
+      <c r="D2" s="28">
+        <v>44</v>
+      </c>
+      <c r="F2" s="94" t="s">
+        <v>621</v>
+      </c>
+      <c r="G2" s="94">
+        <v>242</v>
+      </c>
+      <c r="H2">
+        <f>SUM(Lemons)</f>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="94" t="s">
+        <v>584</v>
+      </c>
+      <c r="B3" s="28">
+        <v>33</v>
+      </c>
+      <c r="C3" s="28">
+        <v>32</v>
+      </c>
+      <c r="D3" s="28">
+        <v>66</v>
+      </c>
+      <c r="F3" s="94" t="s">
+        <v>712</v>
+      </c>
+      <c r="G3" s="94">
+        <v>48.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="94" t="s">
+        <v>582</v>
+      </c>
+      <c r="B4" s="28">
+        <v>45</v>
+      </c>
+      <c r="C4" s="28">
+        <v>50</v>
+      </c>
+      <c r="D4" s="28">
+        <v>44</v>
+      </c>
+      <c r="F4" s="94" t="s">
+        <v>713</v>
+      </c>
+      <c r="G4" s="94">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="94" t="s">
+        <v>708</v>
+      </c>
+      <c r="B5" s="28">
+        <v>34</v>
+      </c>
+      <c r="C5" s="28">
+        <v>32</v>
+      </c>
+      <c r="D5" s="28">
+        <v>22</v>
+      </c>
+      <c r="F5" s="94" t="s">
+        <v>714</v>
+      </c>
+      <c r="G5" s="94">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="94" t="s">
+        <v>585</v>
+      </c>
+      <c r="B6" s="28">
+        <v>21</v>
+      </c>
+      <c r="C6" s="28">
+        <v>26</v>
+      </c>
+      <c r="D6" s="28">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA1000"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -50226,7 +50992,7 @@
       <c r="X1000" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="colorScale" priority="10">
       <colorScale>
@@ -50260,7 +51026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D1199D8-C254-48C0-AC5F-ADDEC91F4A49}">
   <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -50492,7 +51258,7 @@
       <c r="L26" s="37"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{AFE13D69-7C3F-4364-A764-94BD20E9F59C}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{D4312324-D04C-4765-8A3B-1506DE463DAC}"/>
@@ -50503,7 +51269,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD2C2FD5-8379-4925-B2E3-1BBDDF1E9A2D}">
   <dimension ref="A1:L22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -50584,12 +51350,12 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9ADD8E7-B498-4D82-A60B-0B043A12DAA9}">
   <dimension ref="A1:L22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -50908,7 +51674,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B9">
     <sortCondition ref="A2:A9" customList="January,February,March,April,May,June,July,August,September,October,November,December"/>
   </sortState>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="B1:B9">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
       <formula>20000</formula>
@@ -50921,7 +51687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245A1291-890C-4E69-BBCE-61FD758841BF}">
   <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -51315,7 +52081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6891C419-E3F4-4F78-B82D-457603678086}">
   <dimension ref="C2:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -51379,7 +52145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24C003C-206A-4005-AB81-1F886CB6485B}">
   <dimension ref="B3:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -51564,226 +52330,4 @@
   <autoFilter ref="C15:C24" xr:uid="{F24C003C-206A-4005-AB81-1F886CB6485B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4FCD3B0-4BC8-4681-8037-4E058512B5F9}">
-  <dimension ref="B1:J15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="J1" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="85" t="s">
-        <v>686</v>
-      </c>
-      <c r="C2" s="85" t="s">
-        <v>600</v>
-      </c>
-      <c r="D2" s="85" t="s">
-        <v>577</v>
-      </c>
-      <c r="E2" s="85" t="s">
-        <v>624</v>
-      </c>
-      <c r="F2" s="85" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="25">
-        <v>1001</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>604</v>
-      </c>
-      <c r="D3" s="25">
-        <v>70000</v>
-      </c>
-      <c r="E3" s="84">
-        <v>0.1</v>
-      </c>
-      <c r="F3" s="25">
-        <v>7000</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B4" s="25">
-        <v>1002</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>605</v>
-      </c>
-      <c r="D4" s="25">
-        <v>50000</v>
-      </c>
-      <c r="E4" s="84">
-        <v>0.05</v>
-      </c>
-      <c r="F4" s="25">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="25">
-        <v>1003</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>606</v>
-      </c>
-      <c r="D5" s="25">
-        <v>45000</v>
-      </c>
-      <c r="E5" s="84">
-        <v>0</v>
-      </c>
-      <c r="F5" s="25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B6" s="25">
-        <v>1004</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>607</v>
-      </c>
-      <c r="D6" s="25">
-        <v>75000</v>
-      </c>
-      <c r="E6" s="84">
-        <v>0.15</v>
-      </c>
-      <c r="F6" s="25">
-        <v>11250</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B7" s="25">
-        <v>1005</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>623</v>
-      </c>
-      <c r="D7" s="25">
-        <v>55000</v>
-      </c>
-      <c r="E7" s="84">
-        <v>0.05</v>
-      </c>
-      <c r="F7" s="25">
-        <v>2750</v>
-      </c>
-      <c r="G7" t="s">
-        <v>688</v>
-      </c>
-      <c r="H7">
-        <f>MATCH(B4,B2:B7,0)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C8" s="89" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C9" s="87" t="s">
-        <v>687</v>
-      </c>
-      <c r="D9" s="87" t="s">
-        <v>577</v>
-      </c>
-      <c r="E9" s="87" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C10" s="25">
-        <v>1002</v>
-      </c>
-      <c r="D10" s="25">
-        <f>VLOOKUP(C10,B2:F7,MATCH("Sales",B2:F2,0),FALSE)</f>
-        <v>50000</v>
-      </c>
-      <c r="E10" s="88">
-        <f>VLOOKUP(C10,B2:F7,MATCH("Bonus Amount",B2:F2,0),FALSE)</f>
-        <v>2500</v>
-      </c>
-      <c r="G10" t="s">
-        <v>689</v>
-      </c>
-      <c r="H10">
-        <f>MATCH("Sales",B2:F2,0)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="G11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C12" s="86" t="s">
-        <v>691</v>
-      </c>
-      <c r="G12" t="s">
-        <v>688</v>
-      </c>
-      <c r="I12">
-        <f>MATCH(C15,B2:B7,0)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="G13" t="s">
-        <v>689</v>
-      </c>
-      <c r="I13">
-        <f>MATCH("Sales",B2:F2,0)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C14" s="90" t="s">
-        <v>687</v>
-      </c>
-      <c r="D14" s="90" t="s">
-        <v>577</v>
-      </c>
-      <c r="E14" s="90" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C15" s="25">
-        <v>1004</v>
-      </c>
-      <c r="D15" s="25">
-        <f>INDEX(B2:F7,MATCH(C15,B2:B7,0),MATCH("Sales",B2:F2,0))</f>
-        <v>75000</v>
-      </c>
-      <c r="E15" s="25">
-        <f>INDEX(B2:F7,MATCH(C15,B2:B7,0),MATCH("Bonus Amount",B2:F2,0))</f>
-        <v>11250</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10" xr:uid="{A047E17B-A2CA-4FD8-92FF-2040F978D0C4}">
-      <formula1>$B$3:$B$7</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15" xr:uid="{D0E06332-745C-4019-A65E-6A1EF7168DF7}">
-      <formula1>$B$2:$B$7</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>